<commit_message>
feat: additional bindings SNOMED CT et CISIS "Autre acte" sur Procedure.code
Supprime le code NCIT (C25218), remplacé par deux additional bindings
extensibles : SNOMED CT (périmètre repris de procedures-uv-ips, parent
EU Core) pour la demande/report d'acte à des fins internationales, et
CISIS GEN-092.04.13 "Autre acte" en repli si l'acte n'est pas trouvé
dans CCAM ni SNOMED CT.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com> db13728357862959c63aef67f4cadef07d86a200
</commit_message>
<xml_diff>
--- a/nr-doc-core-procedure/ig/StructureDefinition-fr-core-practitioner.xlsx
+++ b/nr-doc-core-procedure/ig/StructureDefinition-fr-core-practitioner.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-03T08:32:23+00:00</t>
+    <t>2026-09-16T15:06:55+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1561,7 +1561,7 @@
     <t>Practitioner.qualification:degree.code.coding:degree</t>
   </si>
   <si>
-    <t>https://mos.esante.gouv.fr/NOS/JDV_J105-EnsembleDiplome-RASS/FHIR/JDV-J105-EnsembleDiplome-RASS|20260223120000</t>
+    <t>https://mos.esante.gouv.fr/NOS/JDV_J105-EnsembleDiplome-RASS/FHIR/JDV-J105-EnsembleDiplome-RASS|20260730120000</t>
   </si>
   <si>
     <t>Practitioner.qualification:degree.code.text</t>
@@ -1715,7 +1715,7 @@
     <t>Compétence acquise par le professionnel (competence) R39 ou Compétence exclusive exercée par le professionnel à titre exclusif (competenceExclusive) R40 ou Diplôme d'études spécialisées complémentaires (DESC)DESCnonQualifian R42 ou Capacité (savoir-faire)de médecine (capaciteSavoirFaire) R43 ou Qualification de praticien adjoint contractuel (qualificationPAC) R44 ou Fonction qualifiée (Synonyme: fonctionQualifiee) R45 ou Droit d'exercice complémentaire (Synonyme: droitExerciceComplementaire) R97 ou Orientation particulière (Synonyme: orientationParticuliere) G13 ou Activité ponctuelle du professionnel de type expertise (attributionParticuliere) G13.</t>
   </si>
   <si>
-    <t>https://mos.esante.gouv.fr/NOS/JDV_J107-EnsembleSavoirFaire-RASS/FHIR/JDV-J107-EnsembleSavoirFaire-RASS|20251222120000</t>
+    <t>https://mos.esante.gouv.fr/NOS/JDV_J107-EnsembleSavoirFaire-RASS/FHIR/JDV-J107-EnsembleSavoirFaire-RASS|20260730120000</t>
   </si>
   <si>
     <t>Practitioner.qualification:savoirFaire.code.text</t>

</xml_diff>